<commit_message>
fix(debug inaccuracy report )
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,33 +435,33 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>440.00</t>
+          <t>660.00</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>320.00</t>
+          <t>440.00</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>178.71</t>
+          <t>690.00</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -481,11 +481,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>660.00</t>
+          <t>240.00</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -501,30 +501,10 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>300.00</t>
+          <t>270.00</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2640.00</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>1100.00</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(revert to older logic )
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,37 +435,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>118</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>660.00</t>
+          <t>440.00</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>440.00</t>
+          <t>880.00</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>690.00</t>
+          <t>270.00</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -481,7 +481,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>240.00</t>
+          <t>80.00</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -491,20 +491,50 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>120.00</t>
+          <t>660.00</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>270.00</t>
+          <t>2640.00</t>
         </is>
       </c>
       <c r="B9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1100.00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>150.00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>160.00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>